<commit_message>
Remove champagne moments, earnest sponsors, S1 GW5 corrected to 2-1 in the sheet copy
Sponsor strip hover no longer shifts layout. Legacy workbook cross-checked: no
recoverable S4 scores or scorers. www.thameslinkhajduci.com added as a redirect.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheet-fixes/thameslink-hajduci-corrected.xlsx
+++ b/sheet-fixes/thameslink-hajduci-corrected.xlsx
@@ -15074,7 +15074,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G6" s="26" t="n">
         <v>5</v>
@@ -15130,7 +15130,7 @@
         <v>3</v>
       </c>
       <c r="F7" s="26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G7" s="26" t="n">
         <v>9</v>

</xml_diff>

<commit_message>
Credit the pitch payer: Isaac is owed, not owing
Money tab Paid formula now adds pitch costs of played games for the season payer
(corrected workbook + report); the site applies the same credit when the sheet
does not, and shows negative balances as money owed to the player.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheet-fixes/thameslink-hajduci-corrected.xlsx
+++ b/sheet-fixes/thameslink-hajduci-corrected.xlsx
@@ -10817,7 +10817,12 @@
       </c>
       <c r="G3" s="33" t="inlineStr">
         <is>
-          <t>Balance owed</t>
+          <t>Balance (+ owes · − is owed)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Paid = transfers logged on Payments + pitch costs of played games in any season this player paid for (row 2). A negative balance means the club owes them.</t>
         </is>
       </c>
     </row>
@@ -10844,7 +10849,7 @@
         <v/>
       </c>
       <c r="F4" s="34">
-        <f>SUMIF(Payments!$B:$B,$A4,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A4,Payments!$C:$C)+IF($A4=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A4=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A4=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G4" s="25">
@@ -10875,7 +10880,7 @@
         <v/>
       </c>
       <c r="F5" s="34">
-        <f>SUMIF(Payments!$B:$B,$A5,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A5,Payments!$C:$C)+IF($A5=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A5=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A5=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G5" s="25">
@@ -10906,7 +10911,7 @@
         <v/>
       </c>
       <c r="F6" s="34">
-        <f>SUMIF(Payments!$B:$B,$A6,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A6,Payments!$C:$C)+IF($A6=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A6=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A6=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G6" s="25">
@@ -10937,7 +10942,7 @@
         <v/>
       </c>
       <c r="F7" s="34">
-        <f>SUMIF(Payments!$B:$B,$A7,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A7,Payments!$C:$C)+IF($A7=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A7=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A7=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G7" s="25">
@@ -10968,7 +10973,7 @@
         <v/>
       </c>
       <c r="F8" s="34">
-        <f>SUMIF(Payments!$B:$B,$A8,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A8,Payments!$C:$C)+IF($A8=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A8=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A8=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G8" s="25">
@@ -10999,7 +11004,7 @@
         <v/>
       </c>
       <c r="F9" s="34">
-        <f>SUMIF(Payments!$B:$B,$A9,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A9,Payments!$C:$C)+IF($A9=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A9=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A9=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G9" s="25">
@@ -11030,7 +11035,7 @@
         <v/>
       </c>
       <c r="F10" s="34">
-        <f>SUMIF(Payments!$B:$B,$A10,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A10,Payments!$C:$C)+IF($A10=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A10=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A10=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G10" s="25">
@@ -11061,7 +11066,7 @@
         <v/>
       </c>
       <c r="F11" s="34">
-        <f>SUMIF(Payments!$B:$B,$A11,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A11,Payments!$C:$C)+IF($A11=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A11=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A11=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G11" s="25">
@@ -11092,7 +11097,7 @@
         <v/>
       </c>
       <c r="F12" s="34">
-        <f>SUMIF(Payments!$B:$B,$A12,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A12,Payments!$C:$C)+IF($A12=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A12=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A12=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G12" s="25">
@@ -11123,7 +11128,7 @@
         <v/>
       </c>
       <c r="F13" s="34">
-        <f>SUMIF(Payments!$B:$B,$A13,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A13,Payments!$C:$C)+IF($A13=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A13=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A13=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G13" s="25">
@@ -11154,7 +11159,7 @@
         <v/>
       </c>
       <c r="F14" s="34">
-        <f>SUMIF(Payments!$B:$B,$A14,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A14,Payments!$C:$C)+IF($A14=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A14=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A14=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G14" s="25">
@@ -11185,7 +11190,7 @@
         <v/>
       </c>
       <c r="F15" s="34">
-        <f>SUMIF(Payments!$B:$B,$A15,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A15,Payments!$C:$C)+IF($A15=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A15=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A15=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G15" s="25">
@@ -11216,7 +11221,7 @@
         <v/>
       </c>
       <c r="F16" s="34">
-        <f>SUMIF(Payments!$B:$B,$A16,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A16,Payments!$C:$C)+IF($A16=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A16=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A16=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G16" s="25">
@@ -11247,7 +11252,7 @@
         <v/>
       </c>
       <c r="F17" s="34">
-        <f>SUMIF(Payments!$B:$B,$A17,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A17,Payments!$C:$C)+IF($A17=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A17=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A17=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G17" s="25">
@@ -11278,7 +11283,7 @@
         <v/>
       </c>
       <c r="F18" s="34">
-        <f>SUMIF(Payments!$B:$B,$A18,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A18,Payments!$C:$C)+IF($A18=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A18=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A18=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G18" s="25">
@@ -11309,7 +11314,7 @@
         <v/>
       </c>
       <c r="F19" s="34">
-        <f>SUMIF(Payments!$B:$B,$A19,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A19,Payments!$C:$C)+IF($A19=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A19=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A19=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G19" s="25">
@@ -11340,7 +11345,7 @@
         <v/>
       </c>
       <c r="F20" s="34">
-        <f>SUMIF(Payments!$B:$B,$A20,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A20,Payments!$C:$C)+IF($A20=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A20=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A20=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G20" s="25">
@@ -11371,7 +11376,7 @@
         <v/>
       </c>
       <c r="F21" s="34">
-        <f>SUMIF(Payments!$B:$B,$A21,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A21,Payments!$C:$C)+IF($A21=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A21=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A21=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G21" s="25">
@@ -11402,7 +11407,7 @@
         <v/>
       </c>
       <c r="F22" s="34">
-        <f>SUMIF(Payments!$B:$B,$A22,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A22,Payments!$C:$C)+IF($A22=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A22=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A22=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G22" s="25">
@@ -11433,7 +11438,7 @@
         <v/>
       </c>
       <c r="F23" s="34">
-        <f>SUMIF(Payments!$B:$B,$A23,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A23,Payments!$C:$C)+IF($A23=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A23=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A23=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G23" s="25">
@@ -11464,7 +11469,7 @@
         <v/>
       </c>
       <c r="F24" s="34">
-        <f>SUMIF(Payments!$B:$B,$A24,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A24,Payments!$C:$C)+IF($A24=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A24=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A24=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G24" s="25">
@@ -11495,7 +11500,7 @@
         <v/>
       </c>
       <c r="F25" s="34">
-        <f>SUMIF(Payments!$B:$B,$A25,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A25,Payments!$C:$C)+IF($A25=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A25=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A25=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G25" s="25">
@@ -11522,7 +11527,7 @@
         <v/>
       </c>
       <c r="F26" s="34">
-        <f>SUMIF(Payments!$B:$B,$A26,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A26,Payments!$C:$C)+IF($A26=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A26=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A26=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G26" s="25">
@@ -11549,7 +11554,7 @@
         <v/>
       </c>
       <c r="F27" s="34">
-        <f>SUMIF(Payments!$B:$B,$A27,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A27,Payments!$C:$C)+IF($A27=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A27=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A27=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G27" s="25">
@@ -11576,7 +11581,7 @@
         <v/>
       </c>
       <c r="F28" s="34">
-        <f>SUMIF(Payments!$B:$B,$A28,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A28,Payments!$C:$C)+IF($A28=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A28=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A28=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G28" s="25">
@@ -11603,7 +11608,7 @@
         <v/>
       </c>
       <c r="F29" s="34">
-        <f>SUMIF(Payments!$B:$B,$A29,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A29,Payments!$C:$C)+IF($A29=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A29=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A29=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G29" s="25">
@@ -11630,7 +11635,7 @@
         <v/>
       </c>
       <c r="F30" s="34">
-        <f>SUMIF(Payments!$B:$B,$A30,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A30,Payments!$C:$C)+IF($A30=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A30=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A30=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G30" s="25">
@@ -11657,7 +11662,7 @@
         <v/>
       </c>
       <c r="F31" s="34">
-        <f>SUMIF(Payments!$B:$B,$A31,Payments!$C:$C)</f>
+        <f>SUMIF(Payments!$B:$B,$A31,Payments!$C:$C)+IF($A31=$B$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;B$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;B$1&amp;"'!$B$13:$U$13")),0),0)+IF($A31=$C$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;C$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;C$1&amp;"'!$B$13:$U$13")),0),0)+IF($A31=$D$2,IFERROR(SUMPRODUCT((INDIRECT("'"&amp;D$1&amp;"'!$B$14:$U$14")&gt;0)*INDIRECT("'"&amp;D$1&amp;"'!$B$13:$U$13")),0),0)</f>
         <v/>
       </c>
       <c r="G31" s="25">

</xml_diff>

<commit_message>
Rename players: Robin -> Robin Watson, Eddie Ringer -> Eddie McLaughlin
Site alias map and bundled extras updated; corrected workbook renames all 23 cells.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheet-fixes/thameslink-hajduci-corrected.xlsx
+++ b/sheet-fixes/thameslink-hajduci-corrected.xlsx
@@ -548,7 +548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B45"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="3" customWidth="1" style="38" min="1" max="1"/>
@@ -556,6 +556,7 @@
     <col width="8.710000000000001" customWidth="1" style="38" min="3" max="26"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="24" customHeight="1" s="38">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -3024,7 +3025,7 @@
     <row r="25" ht="15.75" customHeight="1" s="38">
       <c r="A25" s="23" t="inlineStr">
         <is>
-          <t>Eddie Ringer</t>
+          <t>Eddie McLaughlin</t>
         </is>
       </c>
       <c r="B25" s="27" t="n"/>
@@ -3444,7 +3445,7 @@
     <row r="37" ht="15.75" customHeight="1" s="38">
       <c r="A37" s="23" t="inlineStr">
         <is>
-          <t>Robin</t>
+          <t>Robin Watson</t>
         </is>
       </c>
       <c r="B37" s="27" t="n"/>
@@ -7511,7 +7512,7 @@
     <row r="10">
       <c r="A10" s="23" t="inlineStr">
         <is>
-          <t>Eddie Ringer</t>
+          <t>Eddie McLaughlin</t>
         </is>
       </c>
       <c r="B10" s="27">
@@ -8747,7 +8748,7 @@
     <row r="22" ht="15.75" customHeight="1" s="38">
       <c r="A22" s="23" t="inlineStr">
         <is>
-          <t>Robin</t>
+          <t>Robin Watson</t>
         </is>
       </c>
       <c r="B22" s="27">
@@ -10820,7 +10821,7 @@
           <t>Balance (+ owes · − is owed)</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="0" t="inlineStr">
         <is>
           <t>Paid = transfers logged on Payments + pitch costs of played games in any season this player paid for (row 2). A negative balance means the club owes them.</t>
         </is>
@@ -11046,7 +11047,7 @@
     <row r="11">
       <c r="A11" s="23" t="inlineStr">
         <is>
-          <t>Eddie Ringer</t>
+          <t>Eddie McLaughlin</t>
         </is>
       </c>
       <c r="B11" s="34">
@@ -11418,7 +11419,7 @@
     <row r="23" ht="15.75" customHeight="1" s="38">
       <c r="A23" s="23" t="inlineStr">
         <is>
-          <t>Robin</t>
+          <t>Robin Watson</t>
         </is>
       </c>
       <c r="B23" s="34">
@@ -16180,7 +16181,7 @@
     <row r="25" ht="15.75" customHeight="1" s="38">
       <c r="A25" s="23" t="inlineStr">
         <is>
-          <t>Eddie Ringer</t>
+          <t>Eddie McLaughlin</t>
         </is>
       </c>
       <c r="B25" s="27" t="n"/>
@@ -16696,7 +16697,7 @@
     <row r="37" ht="15.75" customHeight="1" s="38">
       <c r="A37" s="23" t="inlineStr">
         <is>
-          <t>Robin</t>
+          <t>Robin Watson</t>
         </is>
       </c>
       <c r="B37" s="27" t="n"/>
@@ -21258,7 +21259,7 @@
     <row r="25" ht="15.75" customHeight="1" s="38">
       <c r="A25" s="23" t="inlineStr">
         <is>
-          <t>Eddie Ringer</t>
+          <t>Eddie McLaughlin</t>
         </is>
       </c>
       <c r="B25" s="27" t="n"/>
@@ -21740,7 +21741,7 @@
     <row r="37" ht="15.75" customHeight="1" s="38">
       <c r="A37" s="23" t="inlineStr">
         <is>
-          <t>Robin</t>
+          <t>Robin Watson</t>
         </is>
       </c>
       <c r="B37" s="27" t="n"/>
@@ -26350,7 +26351,7 @@
     <row r="25" ht="15.75" customHeight="1" s="38">
       <c r="A25" s="23" t="inlineStr">
         <is>
-          <t>Eddie Ringer</t>
+          <t>Eddie McLaughlin</t>
         </is>
       </c>
       <c r="B25" s="27" t="n"/>
@@ -26866,7 +26867,7 @@
     <row r="37" ht="15.75" customHeight="1" s="38">
       <c r="A37" s="23" t="inlineStr">
         <is>
-          <t>Robin</t>
+          <t>Robin Watson</t>
         </is>
       </c>
       <c r="B37" s="27" t="n"/>
@@ -31490,7 +31491,7 @@
     <row r="25" ht="15.75" customHeight="1" s="38">
       <c r="A25" s="23" t="inlineStr">
         <is>
-          <t>Eddie Ringer</t>
+          <t>Eddie McLaughlin</t>
         </is>
       </c>
       <c r="B25" s="27" t="n"/>
@@ -31998,7 +31999,7 @@
     <row r="37" ht="15.75" customHeight="1" s="38">
       <c r="A37" s="23" t="inlineStr">
         <is>
-          <t>Robin</t>
+          <t>Robin Watson</t>
         </is>
       </c>
       <c r="B37" s="27" t="n"/>
@@ -35897,7 +35898,7 @@
       </c>
       <c r="O10" s="27" t="inlineStr">
         <is>
-          <t>Eddie Ringer</t>
+          <t>Eddie McLaughlin</t>
         </is>
       </c>
       <c r="P10" s="27" t="n"/>
@@ -36608,7 +36609,7 @@
     <row r="25" ht="15.75" customHeight="1" s="38">
       <c r="A25" s="23" t="inlineStr">
         <is>
-          <t>Eddie Ringer</t>
+          <t>Eddie McLaughlin</t>
         </is>
       </c>
       <c r="B25" s="27" t="n"/>
@@ -37128,7 +37129,7 @@
     <row r="37" ht="15.75" customHeight="1" s="38">
       <c r="A37" s="23" t="inlineStr">
         <is>
-          <t>Robin</t>
+          <t>Robin Watson</t>
         </is>
       </c>
       <c r="B37" s="27" t="n"/>
@@ -41740,7 +41741,7 @@
     <row r="25" ht="15.75" customHeight="1" s="38">
       <c r="A25" s="23" t="inlineStr">
         <is>
-          <t>Eddie Ringer</t>
+          <t>Eddie McLaughlin</t>
         </is>
       </c>
       <c r="B25" s="27" t="n"/>
@@ -42274,7 +42275,7 @@
     <row r="37" ht="15.75" customHeight="1" s="38">
       <c r="A37" s="23" t="inlineStr">
         <is>
-          <t>Robin</t>
+          <t>Robin Watson</t>
         </is>
       </c>
       <c r="B37" s="27" t="n"/>
@@ -46946,7 +46947,7 @@
     <row r="25" ht="15.75" customHeight="1" s="38">
       <c r="A25" s="23" t="inlineStr">
         <is>
-          <t>Eddie Ringer</t>
+          <t>Eddie McLaughlin</t>
         </is>
       </c>
       <c r="B25" s="27" t="n"/>
@@ -47456,7 +47457,7 @@
     <row r="37" ht="15.75" customHeight="1" s="38">
       <c r="A37" s="23" t="inlineStr">
         <is>
-          <t>Robin</t>
+          <t>Robin Watson</t>
         </is>
       </c>
       <c r="B37" s="27" t="n"/>
@@ -52062,7 +52063,7 @@
     <row r="25" ht="15.75" customHeight="1" s="38">
       <c r="A25" s="23" t="inlineStr">
         <is>
-          <t>Eddie Ringer</t>
+          <t>Eddie McLaughlin</t>
         </is>
       </c>
       <c r="B25" s="27" t="n"/>
@@ -52492,7 +52493,7 @@
     <row r="37" ht="15.75" customHeight="1" s="38">
       <c r="A37" s="23" t="inlineStr">
         <is>
-          <t>Robin</t>
+          <t>Robin Watson</t>
         </is>
       </c>
       <c r="B37" s="27" t="n"/>

</xml_diff>